<commit_message>
Expand Utilization cheat sheet with locked rules and examples
Add Do/Don't rules, Onyx device÷2 note, validated Washington 33%
and Cumberland ~29% examples, and PDF file tip.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/GSF_Utilization_Columns_and_Math.xlsx
+++ b/GSF_Utilization_Columns_and_Math.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utilization Formula" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cheat Sheet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cheat Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utilization Formula" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,6 +64,12 @@
       <color rgb="00006100"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="13"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -103,7 +109,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -125,11 +131,44 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -173,6 +212,16 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -538,6 +587,330 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GSF Utilization — Cheat Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Locked formula after Washington (33% exact) and Cumberland (~29% close).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>FORMULA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Utilization %  =  COUNT(GSF Job = "Yes")  ÷  (physical sets × Mon–Fri weekdays)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>COLUMNS TO PULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Use</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Dispatching (Roads) / Branch (Onyx)</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Filter to one office</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Assignment Date (Roads) / ticket date (Onyx)</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Filter period; count Mon–Fri → W</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>GSF Job (Roads)</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>COUNT rows where value = Yes → In Field Sets</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>GSF Sent or AFAD Sent (Onyx)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>If device counts (often 2/set): SUM ÷ 2 → In Field Sets. If one row = one set-day: COUNT rows &gt; 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Physical sets S</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Office inventory — not in the export; you supply this</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>STEPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>1. Filter export to office + date range</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>2. In Field Sets = COUNT of GSF Job="Yes" (every job type — Lane Closure, Road Closure, etc. all count)</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>3. W = number of Mondays–Fridays from first to last date in the range</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>4. Sets on Hand = S × W</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>5. Utilization % = In Field Sets ÷ Sets on Hand</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>Do</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Count every job-day with GSF present (GSF Job=Yes or GSF Sent&gt;0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>Do</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Put weekend GSF work in the numerator</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>Do not</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Exclude job types (Manual / Guardian / Lane Closure / Road Closure / etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>Do not</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Add Sat/Sun into W (capacity) — weekdays only</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="25" t="inlineStr">
+        <is>
+          <t>Do not</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Average office % for totals — sum counts, then recompute %</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>VALIDATED EXAMPLES</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Case</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Math → result</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>Washington 9 Sep 2026 · S=6 · 1 day</t>
+        </is>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>2 ÷ (6×1) = 33%  (exact match)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>Cumberland 17–23 Aug 2026 · S=7 · 5 weekdays</t>
+        </is>
+      </c>
+      <c r="B32" s="24" t="inlineStr">
+        <is>
+          <t>10 ÷ (7×5) = 10÷35 ≈ 29%  (close)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>Washington 22–25 Jun 2026 · S=6 · 4 weekdays (Onyx)</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>9 ÷ (6×4) = 9÷24 = 37.5%  (all GSF types)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>FILE TIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="36" customHeight="1">
+      <c r="A36" s="26" t="inlineStr">
+        <is>
+          <t>Roads PDF exports (even column-split) reconstruct cleanly. Prefer PDF or a clean CSV with GSF Job + Assignment Date + Dispatching visible.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A35:B35"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -559,7 +932,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Working rule validated against Washington (~24%), Cumberland (~29% with 7 sets). Count every GSF Job=Yes row — do not filter by Job Type.</t>
+          <t>Working rule validated: Washington Sep 9 = 33% exact; Cumberland ≈ 29% close. COUNT every GSF Job=Yes row — do not filter by Job Type.</t>
         </is>
       </c>
     </row>
@@ -1175,105 +1548,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="70" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Cheat sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Pull</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t>Dispatching (office filter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Assignment Date (period + weekdays)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>GSF Job = Yes (count these rows)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>Physical sets S (from inventory — not in export)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Compute</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>In Field Sets = COUNT(GSF Job = "Yes")</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>W = count of Mon–Fri in the date range</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>Sets on Hand = S × W</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>Utilization % = In Field Sets ÷ Sets on Hand</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>Utilization % = COUNT(GSF Job="Yes") ÷ (physical sets × weekdays)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>